<commit_message>
Docs: Cap nhat Sprint 03 va Sprint 04 Backlog va Tasks vao file Excel Project Plan
</commit_message>
<xml_diff>
--- a/Project Plan Campus Activity Manager (MAUI) (2).xlsx
+++ b/Project Plan Campus Activity Manager (MAUI) (2).xlsx
@@ -11,8 +11,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rủi ro" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 01 backlog" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 02 backlog" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks srpint 01" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks sprint 02" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 03 backlog" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 04 backlog" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks srpint 01" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks sprint 02" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks sprint 03" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks sprint 04" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -24,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -124,6 +128,17 @@
       <color rgb="FFFF0000"/>
       <sz val="13"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -208,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -338,6 +353,19 @@
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -29920,6 +29948,1510 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" style="53" min="1" max="1"/>
+    <col width="14" customWidth="1" style="53" min="2" max="2"/>
+    <col width="32" customWidth="1" style="53" min="3" max="3"/>
+    <col width="12" customWidth="1" style="53" min="4" max="4"/>
+    <col width="55" customWidth="1" style="53" min="5" max="5"/>
+    <col width="18" customWidth="1" style="53" min="6" max="6"/>
+    <col width="20" customWidth="1" style="53" min="7" max="7"/>
+    <col width="80" customWidth="1" style="53" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="63" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="C1" s="63" t="inlineStr">
+        <is>
+          <t>Tên User Story</t>
+        </is>
+      </c>
+      <c r="D1" s="63" t="inlineStr">
+        <is>
+          <t>Task ID</t>
+        </is>
+      </c>
+      <c r="E1" s="63" t="inlineStr">
+        <is>
+          <t>Mô tả công việc</t>
+        </is>
+      </c>
+      <c r="F1" s="63" t="inlineStr">
+        <is>
+          <t>Estimate Time (giờ)</t>
+        </is>
+      </c>
+      <c r="G1" s="63" t="inlineStr">
+        <is>
+          <t>Người phụ trách</t>
+        </is>
+      </c>
+      <c r="H1" s="63" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="61" t="inlineStr">
+        <is>
+          <t>US17</t>
+        </is>
+      </c>
+      <c r="C2" s="62" t="inlineStr">
+        <is>
+          <t>Quét mã QR &amp; Tạo vé QR điểm danh thực tế</t>
+        </is>
+      </c>
+      <c r="D2" s="61" t="inlineStr">
+        <is>
+          <t>T17.1</t>
+        </is>
+      </c>
+      <c r="E2" s="62" t="inlineStr">
+        <is>
+          <t>Xây dựng API xác thực mã QR điểm danh (POST /api/v1/attendance/qr-checkin)</t>
+        </is>
+      </c>
+      <c r="F2" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Đức Mạnh</t>
+        </is>
+      </c>
+      <c r="H2" s="62" t="inlineStr">
+        <is>
+          <t>AC 17.1.1: Tiếp nhận chuỗi QR vé định dạng CAMPUS-ACT:EVT-{id}:STU-{code}:{timestamp}; kiểm tra vé hợp lệ, sự kiện đang mở; ghi nhận điểm danh và cộng điểm rèn luyện.
+AC 17.1.2: Chặn quét trùng lặp (trả về 409 Conflict nếu sinh viên đã điểm danh trước đó).
+AC 17.1.3: Trả về mã lỗi 400 Bad Request nếu mã QR sai định dạng hoặc vé không tồn tại.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>US17</t>
+        </is>
+      </c>
+      <c r="C3" s="62" t="inlineStr">
+        <is>
+          <t>Quét mã QR &amp; Tạo vé QR điểm danh thực tế</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>T17.2</t>
+        </is>
+      </c>
+      <c r="E3" s="62" t="inlineStr">
+        <is>
+          <t>Tích hợp thư viện QRCoder sinh mã QR thật chuẩn PNG/Stream trên mobile app</t>
+        </is>
+      </c>
+      <c r="F3" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" s="61" t="inlineStr">
+        <is>
+          <t>Trần Gia Khánh</t>
+        </is>
+      </c>
+      <c r="H3" s="62" t="inlineStr">
+        <is>
+          <t>AC 17.2.1: Xây dựng IQrCodeService sinh ảnh mã QR độ phân giải cao từ chuỗi vé điện tử.
+AC 17.2.2: Ảnh QR hiển thị sắc nét, tương thích mọi kích thước màn hình, bất kỳ camera điện thoại hay máy quét nào bên ngoài cũng đọc được nội dung vé thực tế.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="61" t="inlineStr">
+        <is>
+          <t>US17</t>
+        </is>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>Quét mã QR &amp; Tạo vé QR điểm danh thực tế</t>
+        </is>
+      </c>
+      <c r="D4" s="61" t="inlineStr">
+        <is>
+          <t>T17.3</t>
+        </is>
+      </c>
+      <c r="E4" s="62" t="inlineStr">
+        <is>
+          <t>Phát triển UI Vé QR điện tử và Màn hình Quét QR chuyên nghiệp (QrScannerPage)</t>
+        </is>
+      </c>
+      <c r="F4" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn An Cương</t>
+        </is>
+      </c>
+      <c r="H4" s="62" t="inlineStr">
+        <is>
+          <t>AC 17.3.1: Màn hình Vé QR hiển thị ảnh QR lớn, tên sự kiện, mã vé, thời gian bắt đầu và hướng dẫn đưa mã cho BTC.
+AC 17.3.2: Màn hình Quét QR (QrScannerPage) có khung ngắm hiện đại, hiệu ứng tia quét laser, hỗ trợ quét ảnh từ thư viện hoặc nhập nhanh mã vé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>US17</t>
+        </is>
+      </c>
+      <c r="C5" s="62" t="inlineStr">
+        <is>
+          <t>Quét mã QR &amp; Tạo vé QR điểm danh thực tế</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>T17.4</t>
+        </is>
+      </c>
+      <c r="E5" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm thử toàn diện chức năng tạo vé và quét điểm danh QR</t>
+        </is>
+      </c>
+      <c r="F5" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H5" s="62" t="inlineStr">
+        <is>
+          <t>AC 17.4.1: Unit tests kiểm thử các trường hợp quét thành công, quét trùng lặp, mã hết hạn hoặc mã rỗng đạt 100% pass.
+AC 17.4.2: Kiểm thử thực tế trên Android Emulator/Device đọc mã QR sinh ra chính xác.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="64" t="inlineStr">
+        <is>
+          <t>Tổng US17</t>
+        </is>
+      </c>
+      <c r="F6" s="64" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>US21</t>
+        </is>
+      </c>
+      <c r="C7" s="62" t="inlineStr">
+        <is>
+          <t>Điểm danh bằng hình ảnh minh chứng &amp; thủ công</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>T21.1</t>
+        </is>
+      </c>
+      <c r="E7" s="62" t="inlineStr">
+        <is>
+          <t>Xây dựng API điểm danh bằng ảnh minh chứng (POST /photo-checkin) và điểm danh thủ công</t>
+        </is>
+      </c>
+      <c r="F7" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Đức Mạnh</t>
+        </is>
+      </c>
+      <c r="H7" s="62" t="inlineStr">
+        <is>
+          <t>AC 21.1.1: Endpoint /api/v1/attendance/photo-checkin tiếp nhận URL/base64 ảnh, ghi chú và mốc thời gian check-in của sinh viên.
+AC 21.1.2: Endpoint /api/v1/attendance/manual cho phép Ban tổ chức/Admin điểm danh bù cho sinh viên không quét được vé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="61" t="inlineStr">
+        <is>
+          <t>US21</t>
+        </is>
+      </c>
+      <c r="C8" s="62" t="inlineStr">
+        <is>
+          <t>Điểm danh bằng hình ảnh minh chứng &amp; thủ công</t>
+        </is>
+      </c>
+      <c r="D8" s="61" t="inlineStr">
+        <is>
+          <t>T21.2</t>
+        </is>
+      </c>
+      <c r="E8" s="62" t="inlineStr">
+        <is>
+          <t>Phát triển giao diện Chụp ảnh điểm danh (PhotoAttendancePage) qua MediaPicker Camera</t>
+        </is>
+      </c>
+      <c r="F8" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn An Cương</t>
+        </is>
+      </c>
+      <c r="H8" s="62" t="inlineStr">
+        <is>
+          <t>AC 21.2.1: Cho phép kích hoạt Camera chụp ảnh thật trực tiếp hoặc chọn ảnh từ thư viện thiết bị.
+AC 21.2.2: Hiển thị ảnh xem trước (Preview), ô nhập ghi chú minh chứng và nút 'Gửi xác nhận điểm danh' nổi bật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>US21</t>
+        </is>
+      </c>
+      <c r="C9" s="62" t="inlineStr">
+        <is>
+          <t>Điểm danh bằng hình ảnh minh chứng &amp; thủ công</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>T21.3</t>
+        </is>
+      </c>
+      <c r="E9" s="62" t="inlineStr">
+        <is>
+          <t>Tích hợp dịch vụ điểm danh ảnh, kết nối API và xử lý lưu trữ ngoại tuyến</t>
+        </is>
+      </c>
+      <c r="F9" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="61" t="inlineStr">
+        <is>
+          <t>Trần Gia Khánh</t>
+        </is>
+      </c>
+      <c r="H9" s="62" t="inlineStr">
+        <is>
+          <t>AC 21.3.1: Tải ảnh và dữ liệu lên API ổn định, hiển thị loading spinner khi tải ảnh.
+AC 21.3.2: Bắt lỗi kết nối mạng linh hoạt, hỗ trợ lưu trữ cục bộ khi mất kết nối.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="61" t="inlineStr">
+        <is>
+          <t>US21</t>
+        </is>
+      </c>
+      <c r="C10" s="62" t="inlineStr">
+        <is>
+          <t>Điểm danh bằng hình ảnh minh chứng &amp; thủ công</t>
+        </is>
+      </c>
+      <c r="D10" s="61" t="inlineStr">
+        <is>
+          <t>T21.4</t>
+        </is>
+      </c>
+      <c r="E10" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm thử chức năng điểm danh bằng ảnh và điểm danh thủ công</t>
+        </is>
+      </c>
+      <c r="F10" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H10" s="62" t="inlineStr">
+        <is>
+          <t>AC 21.4.1: Kiểm thử luồng chụp ảnh, hủy chụp ảnh, upload ảnh thành công và xác nhận điểm danh lưu vào hệ thống.
+AC 21.4.2: Kiểm thử quyền điểm danh thủ công chỉ dành cho vai trò Event Manager/Admin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="64" t="inlineStr">
+        <is>
+          <t>Tổng US21</t>
+        </is>
+      </c>
+      <c r="F11" s="64" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="61" t="inlineStr">
+        <is>
+          <t>US13</t>
+        </is>
+      </c>
+      <c r="C12" s="62" t="inlineStr">
+        <is>
+          <t>Quản lý sự kiện nâng cao &amp; Lịch trình hoạt động</t>
+        </is>
+      </c>
+      <c r="D12" s="61" t="inlineStr">
+        <is>
+          <t>T13.5</t>
+        </is>
+      </c>
+      <c r="E12" s="62" t="inlineStr">
+        <is>
+          <t>Nâng cấp API sự kiện: bổ sung lịch trình (timeline), diễn giả, vị trí và trạng thái điểm danh</t>
+        </is>
+      </c>
+      <c r="F12" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Đức Mạnh</t>
+        </is>
+      </c>
+      <c r="H12" s="62" t="inlineStr">
+        <is>
+          <t>AC 13.5.1: Cập nhật EventDto và CSDL mở rộng: lịch trình chi tiết, danh sách diễn giả, cấu hình check-in.
+AC 13.5.2: API lọc sự kiện theo trạng thái (Sắp diễn ra, Đang diễn ra, Đã kết thúc).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>US13</t>
+        </is>
+      </c>
+      <c r="C13" s="62" t="inlineStr">
+        <is>
+          <t>Quản lý sự kiện nâng cao &amp; Lịch trình hoạt động</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>T13.6</t>
+        </is>
+      </c>
+      <c r="E13" s="62" t="inlineStr">
+        <is>
+          <t>Phát triển giao diện quản lý sự kiện và lịch trình cho Ban tổ chức (EventManagementPage)</t>
+        </is>
+      </c>
+      <c r="F13" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn An</t>
+        </is>
+      </c>
+      <c r="H13" s="62" t="inlineStr">
+        <is>
+          <t>AC 13.6.1: Giao diện quản lý sự kiện phân quyền dành riêng cho Manager/Admin.
+AC 13.6.2: Cho phép chỉnh sửa thời gian check-in, cấu hình số lượng tham gia tối đa và xem danh sách nhanh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="61" t="inlineStr">
+        <is>
+          <t>US13</t>
+        </is>
+      </c>
+      <c r="C14" s="62" t="inlineStr">
+        <is>
+          <t>Quản lý sự kiện nâng cao &amp; Lịch trình hoạt động</t>
+        </is>
+      </c>
+      <c r="D14" s="61" t="inlineStr">
+        <is>
+          <t>T13.7</t>
+        </is>
+      </c>
+      <c r="E14" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm thử tích hợp quản lý sự kiện nâng cao và phân quyền</t>
+        </is>
+      </c>
+      <c r="F14" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H14" s="62" t="inlineStr">
+        <is>
+          <t>AC 13.7.1: Xác thực chỉ Manager/Admin mới có quyền thao tác quản lý sự kiện.
+AC 13.7.2: Dữ liệu sự kiện được cập nhật đồng bộ tức thì trên toàn hệ thống.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="64" t="inlineStr">
+        <is>
+          <t>Tổng US13</t>
+        </is>
+      </c>
+      <c r="F15" s="64" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="61" t="inlineStr">
+        <is>
+          <t>US01</t>
+        </is>
+      </c>
+      <c r="C16" s="62" t="inlineStr">
+        <is>
+          <t>Chi tiết sự kiện toàn diện &amp; Đếm ngược</t>
+        </is>
+      </c>
+      <c r="D16" s="61" t="inlineStr">
+        <is>
+          <t>T01.4</t>
+        </is>
+      </c>
+      <c r="E16" s="62" t="inlineStr">
+        <is>
+          <t>Thiết kế giao diện Chi tiết Sự kiện chuyên nghiệp (EventDetailPage): Banner, Đếm ngược, Diễn giả</t>
+        </is>
+      </c>
+      <c r="F16" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn An Cương</t>
+        </is>
+      </c>
+      <c r="H16" s="62" t="inlineStr">
+        <is>
+          <t>AC 01.4.1: Banner hero cỡ lớn, đồng hồ đếm ngược trực quan tới giờ G.
+AC 01.4.2: Thẻ diễn giả, thông tin địa điểm có bản đồ/chỉ dẫn, thanh tiến độ số lượng đăng ký/sức chứa.
+AC 01.4.3: Các nút thao tác nhanh: Đăng ký tham gia, Xem vé QR điện tử, Điểm danh ảnh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="61" t="inlineStr">
+        <is>
+          <t>US01</t>
+        </is>
+      </c>
+      <c r="C17" s="62" t="inlineStr">
+        <is>
+          <t>Chi tiết sự kiện toàn diện &amp; Đếm ngược</t>
+        </is>
+      </c>
+      <c r="D17" s="61" t="inlineStr">
+        <is>
+          <t>T01.5</t>
+        </is>
+      </c>
+      <c r="E17" s="62" t="inlineStr">
+        <is>
+          <t>Tích hợp logic đếm ngược thời gian thực và điều hướng Shell đa nền tảng</t>
+        </is>
+      </c>
+      <c r="F17" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="61" t="inlineStr">
+        <is>
+          <t>Trần Gia Khánh</t>
+        </is>
+      </c>
+      <c r="H17" s="62" t="inlineStr">
+        <is>
+          <t>AC 01.5.1: Đồng hồ đếm ngược tự động cập nhật mỗi giây, tự chuyển trạng thái khi sự kiện bắt đầu.
+AC 01.5.2: Điều hướng Shell linh hoạt giữa Chi tiết sự kiện &lt;-&gt; Vé QR &lt;-&gt; Điểm danh ảnh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="61" t="inlineStr">
+        <is>
+          <t>US01</t>
+        </is>
+      </c>
+      <c r="C18" s="62" t="inlineStr">
+        <is>
+          <t>Chi tiết sự kiện toàn diện &amp; Đếm ngược</t>
+        </is>
+      </c>
+      <c r="D18" s="61" t="inlineStr">
+        <is>
+          <t>T01.6</t>
+        </is>
+      </c>
+      <c r="E18" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm thử giao diện chi tiết sự kiện trên Android và Windows</t>
+        </is>
+      </c>
+      <c r="F18" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H18" s="62" t="inlineStr">
+        <is>
+          <t>AC 01.6.1: Giao diện hiển thị chuẩn xác, không vỡ layout trên các kích thước màn hình điện thoại và máy tính bảng.
+AC 01.6.2: Kiểm thử thao tác đăng ký sự kiện và mở vé QR mượt mà.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="64" t="inlineStr">
+        <is>
+          <t>Tổng US01</t>
+        </is>
+      </c>
+      <c r="F19" s="64" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="61" t="inlineStr">
+        <is>
+          <t>US23</t>
+        </is>
+      </c>
+      <c r="C20" s="62" t="inlineStr">
+        <is>
+          <t>Cấu hình phương thức điểm danh sự kiện</t>
+        </is>
+      </c>
+      <c r="D20" s="61" t="inlineStr">
+        <is>
+          <t>T23.1</t>
+        </is>
+      </c>
+      <c r="E20" s="62" t="inlineStr">
+        <is>
+          <t>Xây dựng API cấu hình phương thức điểm danh (QR, Ảnh, Thủ công) cho từng sự kiện</t>
+        </is>
+      </c>
+      <c r="F20" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Đức Mạnh</t>
+        </is>
+      </c>
+      <c r="H20" s="62" t="inlineStr">
+        <is>
+          <t>AC 23.1.1: Quản lý các cờ cấu hình AllowQrCheckIn, AllowPhotoCheckIn, AllowManualCheckIn trong Event Model.
+AC 23.1.2: API trả về cấu hình phương thức điểm danh cho client hiển thị phù hợp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="61" t="inlineStr">
+        <is>
+          <t>US23</t>
+        </is>
+      </c>
+      <c r="C21" s="62" t="inlineStr">
+        <is>
+          <t>Cấu hình phương thức điểm danh sự kiện</t>
+        </is>
+      </c>
+      <c r="D21" s="61" t="inlineStr">
+        <is>
+          <t>T23.2</t>
+        </is>
+      </c>
+      <c r="E21" s="62" t="inlineStr">
+        <is>
+          <t>Phát triển UI cấu hình phương thức điểm danh trong form tạo/sửa sự kiện</t>
+        </is>
+      </c>
+      <c r="F21" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn An</t>
+        </is>
+      </c>
+      <c r="H21" s="62" t="inlineStr">
+        <is>
+          <t>AC 23.2.1: Bộ công tắc Switch/Checkbox trực quan cho phép Ban tổ chức bật/tắt từng hình thức điểm danh.
+AC 23.2.2: Hiển thị tooltip giải thích cho từng phương thức điểm danh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="61" t="inlineStr">
+        <is>
+          <t>US23</t>
+        </is>
+      </c>
+      <c r="C22" s="62" t="inlineStr">
+        <is>
+          <t>Cấu hình phương thức điểm danh sự kiện</t>
+        </is>
+      </c>
+      <c r="D22" s="61" t="inlineStr">
+        <is>
+          <t>T23.3</t>
+        </is>
+      </c>
+      <c r="E22" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm thử tính năng bật/tắt phương thức điểm danh</t>
+        </is>
+      </c>
+      <c r="F22" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H22" s="62" t="inlineStr">
+        <is>
+          <t>AC 23.3.1: Khi tắt hình thức điểm danh nào, app sinh viên ẩn tương ứng nút đó trên màn hình chi tiết sự kiện.
+AC 23.3.2: API từ chối nhận request điểm danh nếu phương thức đó đang bị tắt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="64" t="inlineStr">
+        <is>
+          <t>Tổng US23</t>
+        </is>
+      </c>
+      <c r="F23" s="64" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="C24" s="64" t="inlineStr">
+        <is>
+          <t>Tổng thời gian thực hiện sprint 3</t>
+        </is>
+      </c>
+      <c r="F24" s="64" t="n">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:H25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" style="53" min="1" max="1"/>
+    <col width="14" customWidth="1" style="53" min="2" max="2"/>
+    <col width="32" customWidth="1" style="53" min="3" max="3"/>
+    <col width="12" customWidth="1" style="53" min="4" max="4"/>
+    <col width="55" customWidth="1" style="53" min="5" max="5"/>
+    <col width="18" customWidth="1" style="53" min="6" max="6"/>
+    <col width="20" customWidth="1" style="53" min="7" max="7"/>
+    <col width="80" customWidth="1" style="53" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="63" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="C1" s="63" t="inlineStr">
+        <is>
+          <t>Tên User Story</t>
+        </is>
+      </c>
+      <c r="D1" s="63" t="inlineStr">
+        <is>
+          <t>Task ID</t>
+        </is>
+      </c>
+      <c r="E1" s="63" t="inlineStr">
+        <is>
+          <t>Mô tả công việc</t>
+        </is>
+      </c>
+      <c r="F1" s="63" t="inlineStr">
+        <is>
+          <t>Estimate Time (giờ)</t>
+        </is>
+      </c>
+      <c r="G1" s="63" t="inlineStr">
+        <is>
+          <t>Người phụ trách</t>
+        </is>
+      </c>
+      <c r="H1" s="63" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="61" t="inlineStr">
+        <is>
+          <t>US19</t>
+        </is>
+      </c>
+      <c r="C2" s="62" t="inlineStr">
+        <is>
+          <t>Sổ điểm danh &amp; Tính điểm rèn luyện cá nhân</t>
+        </is>
+      </c>
+      <c r="D2" s="61" t="inlineStr">
+        <is>
+          <t>T19.1</t>
+        </is>
+      </c>
+      <c r="E2" s="62" t="inlineStr">
+        <is>
+          <t>Xây dựng API lịch sử điểm danh theo sinh viên (GET /api/v1/attendance/student/{code})</t>
+        </is>
+      </c>
+      <c r="F2" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Đức Mạnh</t>
+        </is>
+      </c>
+      <c r="H2" s="62" t="inlineStr">
+        <is>
+          <t>AC 19.1.1: Trả về danh sách toàn bộ các sự kiện sinh viên đã tham gia kèm hình thức (QR, Ảnh, Thủ công), mốc thời gian và điểm rèn luyện đạt được.
+AC 19.1.2: Tự động tính toán tổng điểm rèn luyện tích lũy và xếp loại rèn luyện.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>US19</t>
+        </is>
+      </c>
+      <c r="C3" s="62" t="inlineStr">
+        <is>
+          <t>Sổ điểm danh &amp; Tính điểm rèn luyện cá nhân</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>T19.2</t>
+        </is>
+      </c>
+      <c r="E3" s="62" t="inlineStr">
+        <is>
+          <t>Thiết kế giao diện Sổ Điểm danh &amp; Điểm rèn luyện cá nhân (AttendanceHistoryPage)</t>
+        </is>
+      </c>
+      <c r="F3" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn An Cương</t>
+        </is>
+      </c>
+      <c r="H3" s="62" t="inlineStr">
+        <is>
+          <t>AC 19.2.1: Card tổng hợp điểm rèn luyện nổi bật, thanh tiến độ rèn luyện (Progress Bar), huy hiệu xếp loại Xuất sắc/Tốt/Khá.
+AC 19.2.2: Danh sách lịch sử sự kiện dạng thẻ, có chip hiển thị phương thức điểm danh (QR / Ảnh / Thủ công) và số điểm cộng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="61" t="inlineStr">
+        <is>
+          <t>US19</t>
+        </is>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>Sổ điểm danh &amp; Tính điểm rèn luyện cá nhân</t>
+        </is>
+      </c>
+      <c r="D4" s="61" t="inlineStr">
+        <is>
+          <t>T19.3</t>
+        </is>
+      </c>
+      <c r="E4" s="62" t="inlineStr">
+        <is>
+          <t>Tích hợp tải lịch sử điểm danh, hỗ trợ lọc theo học kỳ và kéo làm mới (Pull-to-refresh)</t>
+        </is>
+      </c>
+      <c r="F4" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="61" t="inlineStr">
+        <is>
+          <t>Trần Gia Khánh</t>
+        </is>
+      </c>
+      <c r="H4" s="62" t="inlineStr">
+        <is>
+          <t>AC 19.3.1: Tải dữ liệu bất đồng bộ mượt mà, hỗ trợ làm mới danh sách khi kéo xuống.
+AC 19.3.2: Bộ lọc theo năm học/học kỳ giúp sinh viên tra cứu dễ dàng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>US19</t>
+        </is>
+      </c>
+      <c r="C5" s="62" t="inlineStr">
+        <is>
+          <t>Sổ điểm danh &amp; Tính điểm rèn luyện cá nhân</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>T19.4</t>
+        </is>
+      </c>
+      <c r="E5" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm thử chức năng lịch sử điểm danh và tính tổng điểm rèn luyện</t>
+        </is>
+      </c>
+      <c r="F5" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H5" s="62" t="inlineStr">
+        <is>
+          <t>AC 19.4.1: Kiểm tra tính đúng đắn của phép cộng dồn điểm rèn luyện từ các sự kiện.
+AC 19.4.2: Hiển thị EmptyView thân thiện khi sinh viên chưa tham gia sự kiện nào.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="64" t="inlineStr">
+        <is>
+          <t>Tổng US19</t>
+        </is>
+      </c>
+      <c r="F6" s="64" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>US20</t>
+        </is>
+      </c>
+      <c r="C7" s="62" t="inlineStr">
+        <is>
+          <t>Giám sát người tham dự thời gian thực</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>T20.1</t>
+        </is>
+      </c>
+      <c r="E7" s="62" t="inlineStr">
+        <is>
+          <t>Xây dựng API lấy danh sách điểm danh thời gian thực theo sự kiện (GET /event/{eventId})</t>
+        </is>
+      </c>
+      <c r="F7" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Đức Mạnh</t>
+        </is>
+      </c>
+      <c r="H7" s="62" t="inlineStr">
+        <is>
+          <t>AC 20.1.1: Trả về thống kê tổng quan: Số lượng đăng ký, Số lượng đã check-in, Tỷ lệ tham dự (%)
+AC 20.1.2: Danh sách chi tiết từng sinh viên kèm thời điểm điểm danh chính xác.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="61" t="inlineStr">
+        <is>
+          <t>US20</t>
+        </is>
+      </c>
+      <c r="C8" s="62" t="inlineStr">
+        <is>
+          <t>Giám sát người tham dự thời gian thực</t>
+        </is>
+      </c>
+      <c r="D8" s="61" t="inlineStr">
+        <is>
+          <t>T20.2</t>
+        </is>
+      </c>
+      <c r="E8" s="62" t="inlineStr">
+        <is>
+          <t>Phát triển giao diện Giám sát Điểm danh cho Ban tổ chức (EventAttendanceReportPage)</t>
+        </is>
+      </c>
+      <c r="F8" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn An Cương</t>
+        </is>
+      </c>
+      <c r="H8" s="62" t="inlineStr">
+        <is>
+          <t>AC 20.2.1: Thẻ thống kê tỷ lệ tham dự trực quan với vòng tròn tiến độ (Circular Progress).
+AC 20.2.2: Danh sách sinh viên có avatar, MSV, tên, thời gian điểm danh và trạng thái.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>US20</t>
+        </is>
+      </c>
+      <c r="C9" s="62" t="inlineStr">
+        <is>
+          <t>Giám sát người tham dự thời gian thực</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>T20.3</t>
+        </is>
+      </c>
+      <c r="E9" s="62" t="inlineStr">
+        <is>
+          <t>Tích hợp tìm kiếm nhanh sinh viên và điểm danh bổ sung trực tiếp trên danh sách</t>
+        </is>
+      </c>
+      <c r="F9" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn An</t>
+        </is>
+      </c>
+      <c r="H9" s="62" t="inlineStr">
+        <is>
+          <t>AC 20.3.1: Ô tìm kiếm sinh viên theo MSV hoặc Tên phản hồi tức thì.
+AC 20.3.2: Nút điểm danh bù trực tiếp trên danh sách cho sinh viên chưa check-in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="61" t="inlineStr">
+        <is>
+          <t>US20</t>
+        </is>
+      </c>
+      <c r="C10" s="62" t="inlineStr">
+        <is>
+          <t>Giám sát người tham dự thời gian thực</t>
+        </is>
+      </c>
+      <c r="D10" s="61" t="inlineStr">
+        <is>
+          <t>T20.4</t>
+        </is>
+      </c>
+      <c r="E10" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm thử hiệu năng và độ mượt mà khi hiển thị danh sách người tham dự lớn</t>
+        </is>
+      </c>
+      <c r="F10" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H10" s="62" t="inlineStr">
+        <is>
+          <t>AC 20.4.1: Kiểm thử tải danh sách 500+ sinh viên không bị đơ giật UI.
+AC 20.4.2: Tự động cập nhật số liệu khi có sinh viên mới vừa check-in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="64" t="inlineStr">
+        <is>
+          <t>Tổng US20</t>
+        </is>
+      </c>
+      <c r="F11" s="64" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="61" t="inlineStr">
+        <is>
+          <t>US22</t>
+        </is>
+      </c>
+      <c r="C12" s="62" t="inlineStr">
+        <is>
+          <t>Xuất báo cáo điểm danh sự kiện &amp; Tin tức</t>
+        </is>
+      </c>
+      <c r="D12" s="61" t="inlineStr">
+        <is>
+          <t>T22.1</t>
+        </is>
+      </c>
+      <c r="E12" s="62" t="inlineStr">
+        <is>
+          <t>Xây dựng API và Service xuất file báo cáo điểm danh chuẩn CSV UTF-8 có BOM</t>
+        </is>
+      </c>
+      <c r="F12" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Đức Mạnh</t>
+        </is>
+      </c>
+      <c r="H12" s="62" t="inlineStr">
+        <is>
+          <t>AC 22.1.1: Endpoint /api/v1/attendance/event/{eventId}/export tạo file CSV tải về có BOM UTF-8 không lỗi font tiếng Việt trong Microsoft Excel.
+AC 22.1.2: File CSV chứa đầy đủ: STT, Mã sinh viên, Họ tên, Lớp, Thời gian điểm danh, Hình thức, Điểm rèn luyện.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>US22</t>
+        </is>
+      </c>
+      <c r="C13" s="62" t="inlineStr">
+        <is>
+          <t>Xuất báo cáo điểm danh sự kiện &amp; Tin tức</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>T22.2</t>
+        </is>
+      </c>
+      <c r="E13" s="62" t="inlineStr">
+        <is>
+          <t>Tích hợp tính năng lưu và chia sẻ file CSV báo cáo qua Share.RequestAsync()</t>
+        </is>
+      </c>
+      <c r="F13" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="61" t="inlineStr">
+        <is>
+          <t>Trần Gia Khánh</t>
+        </is>
+      </c>
+      <c r="H13" s="62" t="inlineStr">
+        <is>
+          <t>AC 22.2.1: Nhấn nút 'Xuất Báo Cáo CSV' lưu file vào thư mục thiết bị và mở menu chia sẻ (Email, Zalo, Drive).
+AC 22.2.2: Hiển thị thông báo thành công kèm đường dẫn file đã lưu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="61" t="inlineStr">
+        <is>
+          <t>US22</t>
+        </is>
+      </c>
+      <c r="C14" s="62" t="inlineStr">
+        <is>
+          <t>Xuất báo cáo điểm danh sự kiện &amp; Tin tức</t>
+        </is>
+      </c>
+      <c r="D14" s="61" t="inlineStr">
+        <is>
+          <t>T22.3</t>
+        </is>
+      </c>
+      <c r="E14" s="62" t="inlineStr">
+        <is>
+          <t>Phát triển Carousel quảng bá sự kiện nổi bật và chuyên mục Bài viết học đường</t>
+        </is>
+      </c>
+      <c r="F14" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn An Cương</t>
+        </is>
+      </c>
+      <c r="H14" s="62" t="inlineStr">
+        <is>
+          <t>AC 22.3.1: Slide Carousel quảng bá các sự kiện HOT ngay đầu Cổng Sinh viên, tự động cuộn hoặc vuốt mượt mà.
+AC 22.3.2: Danh sách và trang chi tiết Bài viết/Tin tức học đường (ArticleDetailPage) với hình ảnh bìa và nội dung phong phú.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>US22</t>
+        </is>
+      </c>
+      <c r="C15" s="62" t="inlineStr">
+        <is>
+          <t>Xuất báo cáo điểm danh sự kiện &amp; Tin tức</t>
+        </is>
+      </c>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>T22.4</t>
+        </is>
+      </c>
+      <c r="E15" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm thử xuất báo cáo CSV và chuyên mục Tin tức học đường</t>
+        </is>
+      </c>
+      <c r="F15" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H15" s="62" t="inlineStr">
+        <is>
+          <t>AC 22.4.1: Kiểm tra mở file CSV bằng Excel và phần mềm đọc file tiếng Việt hiển thị chính xác các cột.
+AC 22.4.2: Kiểm thử slide sự kiện và chi tiết bài viết hoạt động trơn tru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="64" t="inlineStr">
+        <is>
+          <t>Tổng US22</t>
+        </is>
+      </c>
+      <c r="F16" s="64" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="61" t="inlineStr">
+        <is>
+          <t>US04</t>
+        </is>
+      </c>
+      <c r="C17" s="62" t="inlineStr">
+        <is>
+          <t>Trung tâm Thông báo &amp; Xác nhận Điểm danh tức thì</t>
+        </is>
+      </c>
+      <c r="D17" s="61" t="inlineStr">
+        <is>
+          <t>T04.1</t>
+        </is>
+      </c>
+      <c r="E17" s="62" t="inlineStr">
+        <is>
+          <t>Xây dựng API thông báo sự kiện, xác nhận điểm danh và kênh gửi câu hỏi hỗ trợ (Feedback)</t>
+        </is>
+      </c>
+      <c r="F17" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn Đức Mạnh</t>
+        </is>
+      </c>
+      <c r="H17" s="62" t="inlineStr">
+        <is>
+          <t>AC 04.1.1: API /api/v1/notifications trả về danh sách thông báo sự kiện, nhắc nhở trước giờ G, cộng điểm rèn luyện.
+AC 04.1.2: API /api/v1/feedback tiếp nhận yêu cầu hỗ trợ/góp ý của sinh viên gửi tới quản trị viên.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="61" t="inlineStr">
+        <is>
+          <t>US04</t>
+        </is>
+      </c>
+      <c r="C18" s="62" t="inlineStr">
+        <is>
+          <t>Trung tâm Thông báo &amp; Xác nhận Điểm danh tức thì</t>
+        </is>
+      </c>
+      <c r="D18" s="61" t="inlineStr">
+        <is>
+          <t>T04.2</t>
+        </is>
+      </c>
+      <c r="E18" s="62" t="inlineStr">
+        <is>
+          <t>Thiết kế giao diện Trung tâm Thông báo (NotificationCenterPage) và Modal gửi Hỗ trợ</t>
+        </is>
+      </c>
+      <c r="F18" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn An Cương</t>
+        </is>
+      </c>
+      <c r="H18" s="62" t="inlineStr">
+        <is>
+          <t>AC 04.2.1: Danh sách thông báo phân nhóm trực quan, badge đếm thông báo chưa đọc trên icon chuông.
+AC 04.2.2: Form gửi tin nhắn hỗ trợ trực tiếp tới ban quản trị kèm trạng thái đã giải quyết/đang chờ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="61" t="inlineStr">
+        <is>
+          <t>US04</t>
+        </is>
+      </c>
+      <c r="C19" s="62" t="inlineStr">
+        <is>
+          <t>Trung tâm Thông báo &amp; Xác nhận Điểm danh tức thì</t>
+        </is>
+      </c>
+      <c r="D19" s="61" t="inlineStr">
+        <is>
+          <t>T04.3</t>
+        </is>
+      </c>
+      <c r="E19" s="62" t="inlineStr">
+        <is>
+          <t>Tích hợp thông báo Toast/Alert xác nhận điểm danh tức thì và đánh dấu đã đọc</t>
+        </is>
+      </c>
+      <c r="F19" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" s="61" t="inlineStr">
+        <is>
+          <t>Trần Gia Khánh</t>
+        </is>
+      </c>
+      <c r="H19" s="62" t="inlineStr">
+        <is>
+          <t>AC 04.3.1: Ngay khi điểm danh QR hoặc chụp ảnh thành công, thông báo chúc mừng hiển thị rõ số điểm rèn luyện được cộng.
+AC 04.3.2: Thao tác chạm vào thông báo tự động đánh dấu đã đọc và giảm số badge trên chuông.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="61" t="inlineStr">
+        <is>
+          <t>US04</t>
+        </is>
+      </c>
+      <c r="C20" s="62" t="inlineStr">
+        <is>
+          <t>Trung tâm Thông báo &amp; Xác nhận Điểm danh tức thì</t>
+        </is>
+      </c>
+      <c r="D20" s="61" t="inlineStr">
+        <is>
+          <t>T04.4</t>
+        </is>
+      </c>
+      <c r="E20" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm thử tính năng nhận thông báo, phản hồi hỗ trợ và đánh dấu đã đọc</t>
+        </is>
+      </c>
+      <c r="F20" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H20" s="62" t="inlineStr">
+        <is>
+          <t>AC 04.4.1: Kiểm thử nhận thông báo đúng loại (Nhắc nhở, Điểm danh, Hệ thống).
+AC 04.4.2: Xác minh gửi yêu cầu hỗ trợ thành công và lưu đúng vào cơ sở dữ liệu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="64" t="inlineStr">
+        <is>
+          <t>Tổng US04</t>
+        </is>
+      </c>
+      <c r="F21" s="64" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="61" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+      <c r="C22" s="62" t="inlineStr">
+        <is>
+          <t>Tối ưu UI/UX, Bảng màu Xanh Dương &amp; Đạt chuẩn DoD</t>
+        </is>
+      </c>
+      <c r="D22" s="61" t="inlineStr">
+        <is>
+          <t>TPolish.1</t>
+        </is>
+      </c>
+      <c r="E22" s="62" t="inlineStr">
+        <is>
+          <t>Chuẩn hóa toàn bộ màu sắc (#2563EB), Dark/Light theme, Typography và Shell Navigation</t>
+        </is>
+      </c>
+      <c r="F22" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="61" t="inlineStr">
+        <is>
+          <t>Nguyễn An Cương</t>
+        </is>
+      </c>
+      <c r="H22" s="62" t="inlineStr">
+        <is>
+          <t>AC Polish.1: Toàn bộ các màn hình ứng dụng đồng bộ Bảng màu 1 — Xanh Dương (#2563EB) chuyên nghiệp.
+AC Polish.2: Hỗ trợ hoàn hảo Dark Theme / Light Theme theo cài đặt hệ thống của người dùng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="61" t="inlineStr">
+        <is>
+          <t>Polish</t>
+        </is>
+      </c>
+      <c r="C23" s="62" t="inlineStr">
+        <is>
+          <t>Tối ưu UI/UX, Bảng màu Xanh Dương &amp; Đạt chuẩn DoD</t>
+        </is>
+      </c>
+      <c r="D23" s="61" t="inlineStr">
+        <is>
+          <t>TPolish.2</t>
+        </is>
+      </c>
+      <c r="E23" s="62" t="inlineStr">
+        <is>
+          <t>Tối ưu hiệu năng, loại bỏ hoàn toàn Warning/Error, chạy kiểm thử hồi quy DoD1-DoD6</t>
+        </is>
+      </c>
+      <c r="F23" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="61" t="inlineStr">
+        <is>
+          <t>Vũ Tiến Đạt</t>
+        </is>
+      </c>
+      <c r="H23" s="62" t="inlineStr">
+        <is>
+          <t>AC Polish.3: Biên dịch sạch sẽ 0 Warning, 0 Error trên mọi nền tảng target.
+AC Polish.4: 100% unit tests và integration tests vượt qua thành công, đạt toàn bộ tiêu chuẩn nghiệm thu DoD1–DoD6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="64" t="inlineStr">
+        <is>
+          <t>Tổng Polish</t>
+        </is>
+      </c>
+      <c r="F24" s="64" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" s="64" t="inlineStr">
+        <is>
+          <t>Tổng thời gian thực hiện sprint 4</t>
+        </is>
+      </c>
+      <c r="F25" s="64" t="n">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -35537,8 +37069,6 @@
       <c r="C2" t="n">
         <v>3</v>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>F03</t>
@@ -35562,8 +37092,6 @@
       <c r="C3" t="n">
         <v>2</v>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>F04</t>
@@ -35587,8 +37115,6 @@
       <c r="C4" t="n">
         <v>7</v>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>F05</t>
@@ -35612,8 +37138,6 @@
       <c r="C5" t="n">
         <v>5</v>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>F07</t>
@@ -35637,8 +37161,6 @@
       <c r="C6" t="n">
         <v>4</v>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>F02</t>
@@ -35654,6 +37176,317 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="53" min="1" max="1"/>
+    <col width="75" customWidth="1" style="53" min="2" max="2"/>
+    <col width="12" customWidth="1" style="53" min="3" max="3"/>
+    <col width="12" customWidth="1" style="53" min="6" max="6"/>
+    <col width="14" customWidth="1" style="53" min="7" max="7"/>
+    <col width="20" customWidth="1" style="53" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="H1" s="60" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>US17</t>
+        </is>
+      </c>
+      <c r="B2" s="62" t="inlineStr">
+        <is>
+          <t>As a user, I want to scan a QR code to mark my attendance so that I don’t have to wait in line</t>
+        </is>
+      </c>
+      <c r="C2" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" s="61" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="G2" s="61" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>US21</t>
+        </is>
+      </c>
+      <c r="B3" s="62" t="inlineStr">
+        <is>
+          <t>As an event manager, I want to manually mark attendance for students who cannot scan QR so that records remain accurate</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="61" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="G3" s="61" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="61" t="inlineStr">
+        <is>
+          <t>US23</t>
+        </is>
+      </c>
+      <c r="B4" s="62" t="inlineStr">
+        <is>
+          <t>As an admin, I want to configure attendance methods (QR, RFID, face recognition) so that the system fits different event types</t>
+        </is>
+      </c>
+      <c r="C4" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="F4" s="61" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="G4" s="61" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>US13</t>
+        </is>
+      </c>
+      <c r="B5" s="62" t="inlineStr">
+        <is>
+          <t>As an event manager, I want to create, update information, schedule, send notifications, and manage events so that I can organize campus activities effectively and keep participants informed</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="F5" s="61" t="inlineStr">
+        <is>
+          <t>F05</t>
+        </is>
+      </c>
+      <c r="G5" s="61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="61" t="inlineStr">
+        <is>
+          <t>US01</t>
+        </is>
+      </c>
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>As a student, I want to see all information of an event so that I can decide whether to join and prepare accordingly</t>
+        </is>
+      </c>
+      <c r="C6" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="61" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="G6" s="61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="53" min="1" max="1"/>
+    <col width="75" customWidth="1" style="53" min="2" max="2"/>
+    <col width="12" customWidth="1" style="53" min="3" max="3"/>
+    <col width="12" customWidth="1" style="53" min="6" max="6"/>
+    <col width="14" customWidth="1" style="53" min="7" max="7"/>
+    <col width="20" customWidth="1" style="53" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="H1" s="60" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>US19</t>
+        </is>
+      </c>
+      <c r="B2" s="62" t="inlineStr">
+        <is>
+          <t>As a user, I want to check my attendance history so that I can track my participation in events</t>
+        </is>
+      </c>
+      <c r="C2" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="61" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="G2" s="61" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>US20</t>
+        </is>
+      </c>
+      <c r="B3" s="62" t="inlineStr">
+        <is>
+          <t>As an event manager, I want to see a real-time list of attendees so that I can monitor participation during the event</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" s="61" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="G3" s="61" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="61" t="inlineStr">
+        <is>
+          <t>US22</t>
+        </is>
+      </c>
+      <c r="B4" s="62" t="inlineStr">
+        <is>
+          <t>As an event manager, I want to export attendance reports so that I can evaluate event engagement</t>
+        </is>
+      </c>
+      <c r="C4" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" s="61" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="G4" s="61" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>US04</t>
+        </is>
+      </c>
+      <c r="B5" s="62" t="inlineStr">
+        <is>
+          <t>As a student, I want to have notifications about events that I registered for in the future so that I don’t miss them</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="F5" s="61" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="G5" s="61" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="61" t="inlineStr">
+        <is>
+          <t>US18</t>
+        </is>
+      </c>
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>As a user, I want to receive a confirmation notification after attendance so that I know my presence is recorded</t>
+        </is>
+      </c>
+      <c r="C6" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="61" t="inlineStr">
+        <is>
+          <t>F06</t>
+        </is>
+      </c>
+      <c r="G6" s="61" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>US08</t>
+        </is>
+      </c>
+      <c r="B7" s="62" t="inlineStr">
+        <is>
+          <t>As a user, I want to have a channel to contact with admin when I need support so that I can quickly resolve issues and continue using the system smoothly</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" s="61" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="G7" s="61" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -51445,7 +53278,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -51499,7 +53332,6 @@
       <c r="M1" s="48" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
           <t>US31</t>
@@ -51535,7 +53367,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>US31</t>
@@ -51571,7 +53402,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>US31</t>
@@ -51607,23 +53437,16 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>Tổng US31</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
         <v>8</v>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>US01</t>
@@ -51659,7 +53482,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>US01</t>
@@ -51695,7 +53517,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>US01</t>
@@ -51731,23 +53552,16 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>Tổng US01</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
         <v>7</v>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>US13</t>
@@ -51783,7 +53597,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>US13</t>
@@ -51819,7 +53632,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>US13</t>
@@ -51855,7 +53667,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>US13</t>
@@ -51891,23 +53702,16 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>Tổng US13</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="n">
         <v>22</v>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>US33</t>
@@ -51943,7 +53747,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>US33</t>
@@ -51979,7 +53782,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>US33</t>
@@ -52015,23 +53817,16 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>Tổng US33</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
         <v>12</v>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>US07</t>
@@ -52067,7 +53862,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>US07</t>
@@ -52103,7 +53897,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>US07</t>
@@ -52139,36 +53932,24 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>Tổng US07</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
         <v>11</v>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Tổng thời gian thực hiện sprint 2</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="n">
         <v>60</v>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>